<commit_message>
Upd bg, expand on refresh-centric
</commit_message>
<xml_diff>
--- a/tags.xlsx
+++ b/tags.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
   <si>
     <t xml:space="preserve">Paper</t>
   </si>
@@ -109,12 +109,6 @@
     <t xml:space="preserve">BRC-VL</t>
   </si>
   <si>
-    <t xml:space="preserve">Rowhammer Cache A Last-Level Cache for Low-Overhead Rowhammer Tracking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rowhammer Cache</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rubix Reducing the Overhead of Secure Rowhammer Mitigations via Randomized Line-to-Row Mapping</t>
   </si>
   <si>
@@ -233,6 +227,9 @@
   </si>
   <si>
     <t xml:space="preserve">Orange = Postponed</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -338,7 +335,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -367,6 +364,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -376,6 +377,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -562,7 +567,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.88"/>
@@ -1014,7 +1019,7 @@
       <c r="B11" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D11" s="5" t="n">
@@ -1037,29 +1042,27 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I11" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="I11" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="L11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D12" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1085,41 +1088,39 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J12" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="K12" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="J12" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="L12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C13" s="4" t="s">
+        <v>2025</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="D13" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="H13" s="6" t="n">
         <f aca="false">FALSE()</f>
@@ -1129,25 +1130,25 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J13" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="J13" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="L13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">FALSE()</f>
@@ -1185,7 +1186,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>2025</v>
@@ -1193,37 +1194,37 @@
       <c r="C15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="D15" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="F15" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G15" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="G15" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="J15" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="K15" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="K15" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="L15" s="2"/>
     </row>
@@ -1245,17 +1246,17 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F16" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="F16" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="G16" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H16" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="H16" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="I16" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1389,17 +1390,17 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I19" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="I19" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="J19" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="K19" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K19" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="L19" s="2"/>
     </row>
@@ -1413,13 +1414,13 @@
       <c r="C20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="D20" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="F20" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1433,17 +1434,17 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I20" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="I20" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="J20" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="K20" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="K20" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="L20" s="2"/>
     </row>
@@ -1457,13 +1458,13 @@
       <c r="C21" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="D21" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="F21" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1477,29 +1478,29 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I21" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="I21" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K21" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="L21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D22" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1525,19 +1526,19 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J22" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="K22" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="J22" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="L22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>2025</v>
@@ -1565,13 +1566,13 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I23" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="I23" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="K23" s="6" t="n">
         <f aca="false">FALSE()</f>
@@ -1609,17 +1610,17 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I24" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="I24" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="J24" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="K24" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K24" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="L24" s="2"/>
     </row>
@@ -1653,29 +1654,29 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I25" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="I25" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="J25" s="6" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="K25" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+      <c r="K25" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="L25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D26" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1713,7 +1714,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>2025</v>
@@ -1757,13 +1758,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D28" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1801,13 +1802,13 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D29" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1845,7 +1846,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>2025</v>
@@ -1892,7 +1893,7 @@
         <v>63</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>64</v>
@@ -1961,13 +1962,13 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I32" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="J32" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="I32" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="K32" s="6" t="n">
         <f aca="false">FALSE()</f>
@@ -1976,112 +1977,70 @@
       <c r="L32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="8"/>
+      <c r="C34" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B33" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="8"/>
+      <c r="C35" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="E33" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="F33" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="G33" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H33" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I33" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J33" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="K33" s="6" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L33" s="2"/>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
-      <c r="L34" s="7"/>
-      <c r="M34" s="7"/>
-      <c r="N34" s="7"/>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="7"/>
-      <c r="C35" s="8" t="s">
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
-      <c r="L35" s="7"/>
-      <c r="M35" s="7"/>
-      <c r="N35" s="7"/>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="7"/>
-      <c r="C36" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
-      <c r="L36" s="7"/>
-      <c r="M36" s="7"/>
-      <c r="N36" s="7"/>
-    </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
In the middle of refresh-centric
</commit_message>
<xml_diff>
--- a/tags.xlsx
+++ b/tags.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="72">
   <si>
     <t xml:space="preserve">Paper</t>
   </si>
@@ -94,6 +94,9 @@
     <t xml:space="preserve">Multi-Table Graphene</t>
   </si>
   <si>
+    <t xml:space="preserve">Incomplete</t>
+  </si>
+  <si>
     <t xml:space="preserve">PrIDE Achieving Secure Rowhammer Mitigation with Low-Cost In-DRAM Trackers</t>
   </si>
   <si>
@@ -131,6 +134,9 @@
   </si>
   <si>
     <t xml:space="preserve">Adaptive AI/ML Mitigation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Highly suspicious. Very vague</t>
   </si>
   <si>
     <t xml:space="preserve">CHaRM Checkpointed and Hashed Counters for Flexible and Efficient Rowhammer Mitigation</t>
@@ -269,7 +275,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -292,6 +298,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF6F9D4"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9211E"/>
+        <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
     <fill>
@@ -335,7 +347,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -364,7 +376,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -376,11 +388,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -447,7 +455,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFC9211E"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -843,7 +851,7 @@
       <c r="B7" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="7" t="s">
         <v>23</v>
       </c>
       <c r="D7" s="5" t="n">
@@ -878,17 +886,19 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="L7" s="2"/>
+      <c r="L7" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -926,13 +936,13 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -970,13 +980,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>28</v>
+      <c r="C10" s="4" t="s">
+        <v>29</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1014,13 +1024,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1046,23 +1056,25 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J11" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="K11" s="5" t="b">
+      <c r="J11" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="L11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1088,23 +1100,25 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J12" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="K12" s="5" t="b">
+      <c r="J12" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="L12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D13" s="6" t="n">
         <f aca="false">FALSE()</f>
@@ -1142,13 +1156,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">FALSE()</f>
@@ -1186,13 +1200,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>36</v>
+      <c r="C15" s="7" t="s">
+        <v>37</v>
       </c>
       <c r="D15" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1226,17 +1240,19 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="L15" s="2"/>
+      <c r="L15" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>38</v>
+      <c r="C16" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="D16" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1274,13 +1290,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D17" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1318,13 +1334,13 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D18" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1362,13 +1378,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D19" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1406,13 +1422,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D20" s="6" t="n">
         <f aca="false">FALSE()</f>
@@ -1450,13 +1466,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D21" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1494,13 +1510,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D22" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1538,13 +1554,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D23" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1582,13 +1598,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D24" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1626,13 +1642,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D25" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1670,13 +1686,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D26" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1714,13 +1730,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D27" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1758,13 +1774,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D28" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1802,13 +1818,13 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D29" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1846,13 +1862,13 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D30" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1890,13 +1906,13 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D31" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1934,13 +1950,13 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D32" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -1994,7 +2010,7 @@
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="8"/>
       <c r="C34" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8"/>
@@ -2011,7 +2027,7 @@
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="8"/>
       <c r="C35" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8"/>
@@ -2027,9 +2043,9 @@
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C36" s="11"/>
+        <v>71</v>
+      </c>
+      <c r="C36" s="8"/>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>

</xml_diff>